<commit_message>
Corrected a problem with .env in production
</commit_message>
<xml_diff>
--- a/esempioReale_corretto.xlsx
+++ b/esempioReale_corretto.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Piazza Condini, Romagnano, Trento, Italy</t>
+          <t>Piazza Condini, 38123 Romagnano, Trento, TN, Italia</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Via del Comun, 8, Commezzadura, Trento, Italy</t>
+          <t>Via del Comun, 8, 38020 Commezzadura, TN, Italia</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Viale De Gasperi, 69, Avio, Trento, Italy</t>
+          <t>Viale Alcide Degasperi, 69, 38063 Avio, TN, Italia</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -508,7 +508,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Via 24 Maggio, 115, Lodrone, Trento, Italy</t>
+          <t>Via 24 Maggio, 115, 38089 Lodrone, Storo, TN, Italia</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -527,7 +527,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Strada Provinciale di Seregnano, 4, Civezzano, Trento, Italy</t>
+          <t>Frazione Cogatti, 4, 38045 Seregnano, Civezzano, TN, Italia</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Piazza Fiera, Cles, Trento, Italy</t>
+          <t>Piazza Fiera, 38023 Cles, TN, Italia</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -565,7 +565,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Balbido, 1, 38071, Bleggio Superiore, Trento, Italy</t>
+          <t>Frazione Balbido, 1, 38071 Bleggio Superiore, TN, Italia</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -584,7 +584,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Via Biasi, 1, 38010, San Michele all'Adige, Trento, Italy</t>
+          <t>Via Biasi, 1, 38010 San Michele all'Adige, TN, Italia</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -603,7 +603,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Piazzale Stazione, Mezzolombardo, Trento, Italy</t>
+          <t>Mezzolombardo Stazione FTM, 38017 Mezzolombardo, TN, Italia</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -622,7 +622,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Via Spiazzi, 2, Zivignago, Trento, Italy</t>
+          <t>Via Spiazzi, 2, 38057 Canezza, Pergine Valsugana, TN, Italia</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -641,7 +641,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Corso De Gasperi, 8, Predazzo, Trento, Italy</t>
+          <t>Corso Degasperi, 8, 38037 Predazzo, TN, Italia</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -660,7 +660,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Via Sant'Alessandro, 11, Riva del Garda, Trento, Italy</t>
+          <t>Via S. Alessandro, 11, 38066 Riva del Garda, TN, Italia</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Via dei Laghi, 47, 38060, Tenno, Trento, Italy</t>
+          <t>Via dei Laghi, 47, 38060 Tenno, TN, Italia</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -706,7 +706,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Viale Trento, Rovereto, Trento, Italy</t>
+          <t>Viale Trento, 38068 Rovereto, TN, Italia</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -725,7 +725,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Via Roma, Ospedaletto, Trento, Italy</t>
+          <t>Via Roma, 38050 Ospedaletto, TN, Italia</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -744,7 +744,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Via Alcide De Gasperi, 5, 38096, Terlago, Trento, Italy</t>
+          <t>Via Alcide De Gasperi, 5, 38096 Terlago, TN, Italia</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -763,7 +763,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Piazza de Ciampiedel, Campitello di Fassa, Trento, Italy</t>
+          <t>Piazza Gries, 38032 Canazei, TN, Italia</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -782,7 +782,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Via Temanza, Borgo Valsugana, Trento, Italy</t>
+          <t>Via Temanza, 38051 Borgo Valsugana, TN, Italia</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Piazza de Ciampiedel, Campitello di Fassa, Trento, Italy</t>
+          <t>Piazza San Filippo e Giacomo, 38031 Campitello di Fassa, TN, Italia</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -820,7 +820,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Via Albere, 2, Tenna, Trento, Italy</t>
+          <t>Via Alberè, 2, 38050 Tenna, TN, Italia</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -839,7 +839,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Via della Credenza, Taio, Trento, Italy</t>
+          <t>Via Degli Alpini, 38012 Taio, Predaia, TN, Italia</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -853,36 +853,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IC Trento 7</t>
+          <t>Rovereto 2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Trento, Trento, Italy</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>23</v>
-      </c>
+          <t>Via Alessandro Manzoni, 3, 38068 Rovereto, TN, Italia</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Rovereto 2</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Via Alessandro Manzoni, 3, 38068, Rovereto, Trento, Italy</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>